<commit_message>
update uart function check
</commit_message>
<xml_diff>
--- a/apb_uart_case/teset_plan.xlsx
+++ b/apb_uart_case/teset_plan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ljx62\Documents\Study\github\uvm-study\apb-uart-case\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ljx62\Documents\Study\github\uvm\apb_uart_case\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B96F23F2-24C8-4ED8-9268-607F783635E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EF21E5E-847C-4D5D-912E-C2F1F2255487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4125" yWindow="4185" windowWidth="28800" windowHeight="15435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1740" yWindow="1455" windowWidth="30660" windowHeight="15435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>case name</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -53,9 +53,203 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>tr.rdata[19:0] == 20'd16 
-UVM_ERROR == 0 
-UVM_FATAL == 0</t>
+    <t>apb_rw_reg_test</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>check rw registers corner values</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. CTRL 写入多个 corner values
+2. 读回 CTRL
+3. 只比较有效位 [6:0]
+4. BAUDDIV 写入多个 legal/corner values
+5. 读回 BAUDDIV
+6. 只比较有效位 [19:0]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. read ID register，记录 rdata_before
+2. write 32'hFFFF_FFFF 到同一个地址
+3. read ID register，记录 rdata_after
+4. check rdata_after == rdata_before</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>确认 ID register 是 read-only，不会被 APB write 改掉。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>apb_ro_reg_test</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. 访问未实现地址不会卡死
+2. PSLVERR 仍为 0
+3. 读未实现地址返回 0
+4. 写未实现地址不会破坏 CTRL / BAUDDIV 等已知寄存器</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">READ_value=Write_value
+</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">tr.rdata[19:0] == 20'd16 
+</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. 所有 ID register 都能被 APB read
+2. 对 ID register 写入不会改变其读值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF2C2C2B"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>对若干未实现地址执行 read 
+2. read data 期望为 0 
+3. PSLVERR 期望为 0 
+4. 先写 CTRL / BAUDDIV 为已知值 
+5. 对未实现地址执行 write 
+6. 再读 CTRL / BAUDDIV 
+7. 确认 CTRL / BAUDDIV 没被破坏</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>apb_invalid_addr_test</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>确认读非法地址返回的值为0/don’t care
+写非法地址不会影响正常寄存器的值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CTRL    只保存 [6:0]
+BAUDDIV 只保存 [19:0]
+APB 连续 transaction 没问题
+driver/sequence 不依赖固定值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>apb_safe_reg_random_test</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. 随机的CTRL和BAUDDIV的地址，当随机为BAUDDIV地址的时候写入的值应该大于16
+2. 设置连续读取的次数，这个case是100次
+3. 先写值后读取，判断是否相同</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在进行读写的时候读到的值与写入的值一致</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>APB write TXD register
+ DUT 通过 TXD 串口线发出一帧 UART 数据
+testbench monitor 解析 TXD
+检查发出的 data 等于 APB 写入 data</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. 配置 BAUDDIV 
+2. 使能 CTRL.TXEN 
+3. APB 写 TXD = 8'hA5 
+4. UART TX monitor 从 TXD 上解析出 8'hA5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>uart_tx_basic_test</t>
+  </si>
+  <si>
+    <t>basic tx function</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>uart_tx_multi_data_test</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. 配置 BAUDDIV 
+2. 使能 CTRL.TXEN 
+3. APB 将队列数据写入到TXD
+4. UART TX monitor 从 TXD 上解析出 队列中的所有数据</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>连续写数据正常
+TXD的发送功能正常</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>连续发送功能正常</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>uart_rx_basic_test</t>
+  </si>
+  <si>
+    <t>基本的接收功能正常</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. 配 BAUDDIV
+2. 使能 RX
+3. 驱动 RXD = 8'h5A
+4. poll STAT[1] RX buffer full
+5. APB read RXD register
+6. check rdata[7:0] == 8'h5A
+7. 读完 RXD 写STAT[1]为1 清除</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RXD寄存器能够读取到5A
+写STAT[1]为1清除</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>uart_tx_multi_data_test</t>
+  </si>
+  <si>
+    <t>连续接收功能正常</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. 配 BAUDDIV
+2. 使能 RX
+3. 驱动 RXD赋值队列
+4. poll STAT[1] RX buffer full
+5. APB read RXD register
+6. check rdata[7:0] == 8'h5A
+7. 读完 RXD 写STAT[1]为1 清除</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RXD寄存器能够读取到队列值
+写STAT[1]能清楚full</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -63,7 +257,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -73,6 +267,30 @@
     </font>
     <font>
       <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF2C2C2B"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF2C2C2B"/>
       <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
@@ -99,13 +317,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -387,10 +611,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.75" style="1" customWidth="1"/>
     <col min="2" max="2" width="30.375" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="96.125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="55.875" style="1" bestFit="1" customWidth="1"/>
@@ -422,7 +646,119 @@
         <v>6</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="85.5" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
         <v>7</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="57" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="99.75" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="57" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="57" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="99.75" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="99.75" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>